<commit_message>
Update BOM with cable and potentiometer
</commit_message>
<xml_diff>
--- a/docs/bom/InfraRedFox Mini - Bill of Materials.xlsx
+++ b/docs/bom/InfraRedFox Mini - Bill of Materials.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30502"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="506" documentId="11_924858E5C0DEB8026F15A6DB943E8C1851038383" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B953A51A-064C-4E5C-B71A-BA9E3CAF6A23}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{C8A2E239-40F8-47FB-8A3F-6DC80D47371C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="70">
   <si>
     <t>InfraredFox Mini - Bill of Materials</t>
   </si>
@@ -219,13 +219,22 @@
     <t>Marks the yellow safety boundary used during the demonstration</t>
   </si>
   <si>
-    <t>IR sensor extension cable-TBD</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Extension cable for the long-range IR sensor. Cable type and required length to be confirmed after hardware setup.</t>
+    <t>SKX cable, 2x0.75mm², 5m, white</t>
+  </si>
+  <si>
+    <t>Biltema</t>
+  </si>
+  <si>
+    <t>35-432</t>
+  </si>
+  <si>
+    <t>Extension cable for the long-range IR sensor, allowing flexible sensor placement in the prototype.</t>
+  </si>
+  <si>
+    <t>Trimmer pot 3386P 10k (103) with knob</t>
+  </si>
+  <si>
+    <t>Adjust the contrast of the LCD display.</t>
   </si>
   <si>
     <t>Shipping</t>
@@ -305,7 +314,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -321,12 +330,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -374,12 +377,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -426,16 +423,22 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -753,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:G36"/>
+  <dimension ref="A2:G37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
@@ -766,41 +769,41 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="23.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
     </row>
     <row r="3" spans="1:7" ht="23.25">
       <c r="D3" s="1"/>
     </row>
     <row r="4" spans="1:7" ht="15.75">
-      <c r="A4" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="A4" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
     </row>
     <row r="5" spans="1:7" ht="15.75">
       <c r="B5" s="4"/>
       <c r="C5" s="3"/>
-      <c r="D5" s="8"/>
-      <c r="F5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="F5" s="5"/>
     </row>
     <row r="6" spans="1:7" ht="15.75">
       <c r="B6" s="4"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="8"/>
-      <c r="F6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="F6" s="5"/>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1">
       <c r="B7" s="4"/>
@@ -808,21 +811,21 @@
       <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="10"/>
+      <c r="E8" s="10"/>
+      <c r="F8" s="10"/>
+      <c r="G8" s="10"/>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1">
       <c r="A9" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="7" t="s">
         <v>4</v>
       </c>
     </row>
@@ -830,7 +833,7 @@
       <c r="A10" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="7" t="s">
         <v>6</v>
       </c>
     </row>
@@ -838,7 +841,7 @@
       <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="7" t="s">
         <v>8</v>
       </c>
     </row>
@@ -846,7 +849,7 @@
       <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="7">
         <v>1</v>
       </c>
       <c r="G12" s="4"/>
@@ -855,425 +858,456 @@
       <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="14">
+      <c r="B13" s="12">
         <f>SUM(B14/B12)</f>
-        <v>657.11999999999989</v>
+        <v>703.03999999999985</v>
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="15">
-        <f>SUM(C20:C36,D20:D36)</f>
-        <v>657.11999999999989</v>
+      <c r="B14" s="13">
+        <f>SUM(C20:C37,D20:D37)</f>
+        <v>703.03999999999985</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="15" customHeight="1"/>
     <row r="19" spans="1:7" s="2" customFormat="1" ht="31.5" customHeight="1">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="G19" s="17" t="s">
+      <c r="G19" s="15" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="48" customHeight="1">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="16">
+      <c r="C20" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D20" s="24">
+      <c r="D20" s="22">
         <v>87.2</v>
       </c>
-      <c r="E20" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F20" s="20">
+      <c r="E20" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F20" s="18">
         <v>41024158</v>
       </c>
-      <c r="G20" s="19" t="s">
+      <c r="G20" s="17" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30.75">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B21" s="19" t="s">
+      <c r="B21" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C21" s="16">
+      <c r="C21" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D21" s="24">
+      <c r="D21" s="22">
         <v>55.2</v>
       </c>
-      <c r="E21" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F21" s="21">
+      <c r="E21" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F21" s="19">
         <v>10160840</v>
       </c>
-      <c r="G21" s="19" t="s">
+      <c r="G21" s="17" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="29.25" customHeight="1">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="C22" s="16">
+      <c r="C22" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D22" s="24">
+      <c r="D22" s="22">
         <v>22.4</v>
       </c>
-      <c r="E22" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" s="21">
+      <c r="E22" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" s="19">
         <v>41022181</v>
       </c>
-      <c r="G22" s="19" t="s">
+      <c r="G22" s="17" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="45.75">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="14" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C23" s="16">
+      <c r="C23" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="22">
         <v>36</v>
       </c>
-      <c r="E23" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F23" s="21">
+      <c r="E23" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="19">
         <v>41003181</v>
       </c>
-      <c r="G23" s="19" t="s">
+      <c r="G23" s="17" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30.75">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B24" s="19" t="s">
+      <c r="B24" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C24" s="16">
+      <c r="C24" s="14">
         <f>ROUNDUP($B$12/2,0)</f>
         <v>1</v>
       </c>
-      <c r="D24" s="24">
+      <c r="D24" s="22">
         <v>8</v>
       </c>
-      <c r="E24" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" s="21">
+      <c r="E24" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F24" s="19">
         <v>40307023</v>
       </c>
-      <c r="G24" s="19" t="s">
+      <c r="G24" s="17" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30.75">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="B25" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="16">
+      <c r="C25" s="14">
         <f>ROUNDUP($B$12/6,0)</f>
         <v>1</v>
       </c>
-      <c r="D25" s="24">
+      <c r="D25" s="22">
         <v>9.6</v>
       </c>
-      <c r="E25" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F25" s="21">
+      <c r="E25" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F25" s="19">
         <v>40307031</v>
       </c>
-      <c r="G25" s="19" t="s">
+      <c r="G25" s="17" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30.75">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B26" s="19" t="s">
+      <c r="B26" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C26" s="16">
+      <c r="C26" s="14">
         <f>ROUNDUP($B$12/2,0)</f>
         <v>1</v>
       </c>
-      <c r="D26" s="24">
+      <c r="D26" s="22">
         <v>8</v>
       </c>
-      <c r="E26" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" s="21">
+      <c r="E26" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" s="19">
         <v>40307020</v>
       </c>
-      <c r="G26" s="19" t="s">
+      <c r="G26" s="17" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30.75">
-      <c r="A27" s="16" t="s">
+      <c r="A27" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="19" t="s">
+      <c r="B27" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="16">
+      <c r="C27" s="14">
         <f>ROUNDUP(($B$12*3)/10,0)</f>
         <v>1</v>
       </c>
-      <c r="D27" s="24">
+      <c r="D27" s="22">
         <v>8</v>
       </c>
-      <c r="E27" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F27" s="21">
+      <c r="E27" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F27" s="19">
         <v>40810233</v>
       </c>
-      <c r="G27" s="19" t="s">
+      <c r="G27" s="17" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30.75">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C28" s="16">
+      <c r="C28" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D28" s="24">
+      <c r="D28" s="22">
         <v>14.4</v>
       </c>
-      <c r="E28" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F28" s="21">
+      <c r="E28" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F28" s="19">
         <v>41015713</v>
       </c>
-      <c r="G28" s="19" t="s">
+      <c r="G28" s="17" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30.75">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B29" s="19" t="s">
+      <c r="B29" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="16">
+      <c r="C29" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D29" s="24">
+      <c r="D29" s="22">
         <v>95.2</v>
       </c>
-      <c r="E29" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F29" s="21">
+      <c r="E29" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29" s="19">
         <v>41015028</v>
       </c>
-      <c r="G29" s="19" t="s">
+      <c r="G29" s="17" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="42" customHeight="1">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="19" t="s">
+      <c r="B30" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D30" s="24">
+      <c r="D30" s="22">
         <v>119.2</v>
       </c>
-      <c r="E30" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F30" s="21">
+      <c r="E30" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F30" s="19">
         <v>41017035</v>
       </c>
-      <c r="G30" s="19" t="s">
+      <c r="G30" s="17" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="30.75">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="19" t="s">
+      <c r="B31" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D31" s="24">
+      <c r="D31" s="22">
         <v>95.2</v>
       </c>
-      <c r="E31" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F31" s="21">
+      <c r="E31" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F31" s="19">
         <v>41037104</v>
       </c>
-      <c r="G31" s="19" t="s">
+      <c r="G31" s="17" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="30.75">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="19" t="s">
+      <c r="B32" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="C32" s="16">
+      <c r="C32" s="14">
         <f>ROUNDUP($B$12/2,0)</f>
         <v>1</v>
       </c>
-      <c r="D32" s="24">
+      <c r="D32" s="22">
         <v>8.8000000000000007</v>
       </c>
-      <c r="E32" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F32" s="21">
+      <c r="E32" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F32" s="19">
         <v>41024494</v>
       </c>
-      <c r="G32" s="19" t="s">
+      <c r="G32" s="17" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="45.75">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B33" s="19" t="s">
+      <c r="B33" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C33" s="16">
+      <c r="C33" s="14">
         <f>$B$12</f>
         <v>1</v>
       </c>
-      <c r="D33" s="24">
+      <c r="D33" s="22">
         <v>39.92</v>
       </c>
-      <c r="E33" s="16" t="s">
+      <c r="E33" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="F33" s="21" t="s">
+      <c r="F33" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="G33" s="19" t="s">
+      <c r="G33" s="17" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:7" s="12" customFormat="1" ht="30.75">
+    <row r="34" spans="1:7" s="10" customFormat="1" ht="30.75">
       <c r="A34" s="25" t="s">
         <v>29</v>
       </c>
       <c r="B34" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="C34" s="25"/>
-      <c r="D34" s="27"/>
+      <c r="C34" s="25">
+        <f>$B$12</f>
+        <v>1</v>
+      </c>
+      <c r="D34" s="27">
+        <v>31.92</v>
+      </c>
       <c r="E34" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="F34" s="28"/>
+      <c r="F34" s="28" t="s">
+        <v>63</v>
+      </c>
       <c r="G34" s="26" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" s="16"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="19"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="30.75">
+      <c r="A35" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="14">
+        <f>$B$12</f>
+        <v>1</v>
+      </c>
+      <c r="D35" s="22">
+        <v>12</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F35" s="18">
+        <v>33860103</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="16" t="s">
-        <v>64</v>
-      </c>
-      <c r="B36" s="23" t="s">
-        <v>65</v>
-      </c>
-      <c r="C36" s="16">
-        <v>1</v>
-      </c>
-      <c r="D36" s="24">
+      <c r="A36" s="14"/>
+      <c r="B36" s="17"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="22"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="17"/>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="14">
+        <v>1</v>
+      </c>
+      <c r="D37" s="22">
         <v>35</v>
       </c>
-      <c r="E36" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="F36" s="16"/>
-      <c r="G36" s="19" t="s">
-        <v>66</v>
+      <c r="E37" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="F37" s="14"/>
+      <c r="G37" s="17" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1296,6 +1330,8 @@
     <hyperlink ref="F32" r:id="rId12" display="41024494" xr:uid="{C72CC122-5795-4574-94B5-55EBD66D1091}"/>
     <hyperlink ref="F33" r:id="rId13" xr:uid="{2DECE53B-D13B-40CF-91FC-E068B5070AC8}"/>
     <hyperlink ref="F30" r:id="rId14" display="41017035" xr:uid="{5E1FED99-2BA4-40F2-8DCD-A1E622389DA1}"/>
+    <hyperlink ref="F34" r:id="rId15" xr:uid="{2673DF96-8935-454E-BB53-94B00E115EC2}"/>
+    <hyperlink ref="F35" r:id="rId16" display="33860103" xr:uid="{311C4A35-5F36-443B-9FFB-3847C2EBBE7E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>